<commit_message>
Update Fossil In-Transit and Replenishment data files
</commit_message>
<xml_diff>
--- a/data/input/Fossil Replenishment/In-Transit_Open_PO_Fossil.xlsx
+++ b/data/input/Fossil Replenishment/In-Transit_Open_PO_Fossil.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\Fossil Replenishment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFE15CED-F7A8-42D5-AA61-D343C7215E71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBD007C1-C26B-49C5-B6F2-0ECB1C5612CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7D8DA65D-B779-44B4-89F3-D67DE71DDA05}"/>
   </bookViews>
@@ -1505,7 +1505,7 @@
     <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.88671875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.88671875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.21875" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
Add In-Transit file to preload cache, update with April POs
</commit_message>
<xml_diff>
--- a/data/input/Fossil Replenishment/In-Transit_Open_PO_Fossil.xlsx
+++ b/data/input/Fossil Replenishment/In-Transit_Open_PO_Fossil.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\Fossil Replenishment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBD007C1-C26B-49C5-B6F2-0ECB1C5612CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{921BE8C6-FCC2-4D45-A59F-2F0E8F02938C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7D8DA65D-B779-44B4-89F3-D67DE71DDA05}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AA$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AA$324</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1517,7 +1517,7 @@
     <col min="15" max="15" width="6" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="5.33203125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="9" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17.88671875" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="14.109375" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="13.6640625" bestFit="1" customWidth="1"/>
@@ -26736,7 +26736,6 @@
       <c r="AA324" s="15"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA1" xr:uid="{6BB0EA74-04A4-4B1E-92E9-B9F100D395D0}"/>
   <conditionalFormatting sqref="J1">
     <cfRule type="duplicateValues" dxfId="3" priority="1"/>
     <cfRule type="duplicateValues" dxfId="2" priority="2"/>

</xml_diff>